<commit_message>
More restructuring the repo and adding and updating files.
</commit_message>
<xml_diff>
--- a/answers_for_interviews/InverviewPrepGrid.xlsx
+++ b/answers_for_interviews/InverviewPrepGrid.xlsx
@@ -5,15 +5,15 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\DakotaStaubach\2026\ComputerScience\CrackingTheCodingInterview\b_V_BehvarioralQuestions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\DakotaStaubach\2026\ComputerScience\CrackingTheCodingInterview\answers_for_interviews\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5513C467-A675-498D-95CD-07C8A55CF85A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EFB1E1BA-4961-4FD1-B5CA-E5BDBE184224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-68" yWindow="8902" windowWidth="21796" windowHeight="13875" xr2:uid="{5A3B6A0C-714A-4120-97EC-1803310A997D}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Resume Responses" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,10 +35,89 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+  <si>
+    <t>CommonQuestions</t>
+  </si>
+  <si>
+    <t>Swipe</t>
+  </si>
+  <si>
+    <t>Challenges</t>
+  </si>
+  <si>
+    <t>Mistakes/Failures</t>
+  </si>
+  <si>
+    <t>Enjoyed</t>
+  </si>
+  <si>
+    <t>Leadership</t>
+  </si>
+  <si>
+    <t>Conflicts</t>
+  </si>
+  <si>
+    <t>What I'd Do Differently</t>
+  </si>
+  <si>
+    <t>Parallel &amp; Distributed Networking</t>
+  </si>
+  <si>
+    <t>Database Management</t>
+  </si>
+  <si>
+    <t>Machine Learning</t>
+  </si>
+  <si>
+    <t>Target Repack Merchandising Sort &amp; Stock</t>
+  </si>
+  <si>
+    <t>BJ's Restaurant &amp; Brewhouse</t>
+  </si>
+  <si>
+    <t>Army National Guard</t>
+  </si>
+  <si>
+    <t>Habitat for Humanity's</t>
+  </si>
+  <si>
+    <t>Target</t>
+  </si>
+  <si>
+    <t>Quiktrip</t>
+  </si>
+  <si>
+    <t>AI Policy &amp; Regulations Map</t>
+  </si>
+  <si>
+    <t>Technical Decisions</t>
+  </si>
+  <si>
+    <t>Choices of Technology</t>
+  </si>
+  <si>
+    <t>Graphics Design</t>
+  </si>
+  <si>
+    <t>Scaling the Project</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -54,7 +133,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -62,12 +141,140 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -402,9 +609,294 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC179D58-4195-4282-994F-216C626D420C}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:AA11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="27" width="50.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:27" s="11" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="L1" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="M1" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="6"/>
+      <c r="Q1" s="6"/>
+      <c r="R1" s="6"/>
+      <c r="S1" s="6"/>
+      <c r="T1" s="5"/>
+      <c r="U1" s="5"/>
+      <c r="V1" s="5"/>
+      <c r="W1" s="5"/>
+      <c r="X1" s="5"/>
+      <c r="Y1" s="5"/>
+      <c r="Z1" s="5"/>
+      <c r="AA1" s="5"/>
+    </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="9"/>
+      <c r="N2" s="9"/>
+      <c r="O2" s="9"/>
+      <c r="P2" s="9"/>
+      <c r="Q2" s="9"/>
+      <c r="R2" s="9"/>
+      <c r="S2" s="9"/>
+      <c r="T2" s="10"/>
+      <c r="U2" s="10"/>
+      <c r="V2" s="10"/>
+      <c r="W2" s="10"/>
+      <c r="X2" s="10"/>
+      <c r="Y2" s="10"/>
+      <c r="Z2" s="10"/>
+      <c r="AA2" s="10"/>
+    </row>
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
+      <c r="Q3" s="3"/>
+      <c r="R3" s="3"/>
+      <c r="S3" s="3"/>
+      <c r="T3" s="2"/>
+      <c r="U3" s="2"/>
+      <c r="V3" s="2"/>
+      <c r="W3" s="2"/>
+      <c r="X3" s="2"/>
+      <c r="Y3" s="2"/>
+      <c r="Z3" s="2"/>
+      <c r="AA3" s="2"/>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3"/>
+      <c r="T4" s="2"/>
+      <c r="U4" s="2"/>
+      <c r="V4" s="2"/>
+      <c r="W4" s="2"/>
+      <c r="X4" s="2"/>
+      <c r="Y4" s="2"/>
+      <c r="Z4" s="2"/>
+      <c r="AA4" s="2"/>
+    </row>
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="3"/>
+      <c r="O5" s="3"/>
+      <c r="P5" s="3"/>
+      <c r="Q5" s="3"/>
+      <c r="R5" s="3"/>
+      <c r="S5" s="3"/>
+      <c r="T5" s="2"/>
+      <c r="U5" s="2"/>
+      <c r="V5" s="2"/>
+      <c r="W5" s="2"/>
+      <c r="X5" s="2"/>
+      <c r="Y5" s="2"/>
+      <c r="Z5" s="2"/>
+      <c r="AA5" s="2"/>
+    </row>
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
+      <c r="H6" s="13"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+      <c r="L6" s="3"/>
+      <c r="M6" s="3"/>
+      <c r="N6" s="3"/>
+      <c r="O6" s="3"/>
+      <c r="P6" s="3"/>
+      <c r="Q6" s="3"/>
+      <c r="R6" s="3"/>
+      <c r="S6" s="3"/>
+      <c r="T6" s="2"/>
+      <c r="U6" s="2"/>
+      <c r="V6" s="2"/>
+      <c r="W6" s="2"/>
+      <c r="X6" s="2"/>
+      <c r="Y6" s="2"/>
+      <c r="Z6" s="2"/>
+      <c r="AA6" s="2"/>
+    </row>
+    <row r="7" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="13"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="4"/>
+      <c r="M7" s="4"/>
+      <c r="N7" s="4"/>
+      <c r="O7" s="4"/>
+      <c r="P7" s="4"/>
+      <c r="Q7" s="4"/>
+      <c r="R7" s="4"/>
+      <c r="S7" s="4"/>
+      <c r="T7" s="1"/>
+      <c r="U7" s="1"/>
+      <c r="V7" s="1"/>
+      <c r="W7" s="1"/>
+      <c r="X7" s="1"/>
+      <c r="Y7" s="1"/>
+      <c r="Z7" s="1"/>
+      <c r="AA7" s="1"/>
+    </row>
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="2"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+    </row>
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A9" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="16"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="16"/>
+    </row>
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A10" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+    </row>
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>